<commit_message>
Stabilize COA PDF rendering and update branding
</commit_message>
<xml_diff>
--- a/src/JinZhaoYi.GasQcDataLoader/templates/COA(小卡).xlsx
+++ b/src/JinZhaoYi.GasQcDataLoader/templates/COA(小卡).xlsx
@@ -684,24 +684,26 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
+            <a:defRPr sz="1200"/>
           </a:pPr>
           <a:r>
             <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:rPr>
             <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+          <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
             <a:solidFill>
               <a:srgbClr val="000000"/>
             </a:solidFill>
-            <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-            <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+            <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+            <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+            <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
@@ -709,7 +711,7 @@
             <a:lnSpc>
               <a:spcPts val="2000"/>
             </a:lnSpc>
-            <a:defRPr sz="1000"/>
+            <a:defRPr sz="1200"/>
           </a:pPr>
           <a:r>
             <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -717,11 +719,19 @@
                 <a:srgbClr val="000000"/>
               </a:solidFill>
               <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
             </a:rPr>
             <a:t>New-Fast Technology Co., LTD</a:t>
           </a:r>
+          <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:pPr algn="l" rtl="0">
@@ -902,24 +912,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -927,7 +939,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -935,11 +947,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -1065,24 +1085,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -1090,7 +1112,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -1098,11 +1120,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -1228,24 +1258,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -1253,7 +1285,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -1261,28 +1293,18 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
-              <a:t>New-Fast Technology Co., LT</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
-              </a:rPr>
-              <a:t>D</a:t>
+              <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:cs typeface="Times New Roman"/>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -1409,24 +1431,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -1434,7 +1458,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -1442,11 +1466,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -1572,24 +1604,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -1597,7 +1631,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -1605,11 +1639,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -1735,24 +1777,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -1760,7 +1804,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -1768,11 +1812,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -1898,24 +1950,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -1923,7 +1977,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -1931,11 +1985,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -2061,24 +2123,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -2086,7 +2150,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -2094,11 +2158,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -2169,24 +2241,26 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
+            <a:defRPr sz="1200"/>
           </a:pPr>
           <a:r>
             <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:rPr>
             <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
           </a:r>
-          <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+          <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
             <a:solidFill>
               <a:srgbClr val="000000"/>
             </a:solidFill>
-            <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-            <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+            <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+            <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+            <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
@@ -2194,7 +2268,7 @@
             <a:lnSpc>
               <a:spcPts val="2000"/>
             </a:lnSpc>
-            <a:defRPr sz="1000"/>
+            <a:defRPr sz="1200"/>
           </a:pPr>
           <a:r>
             <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -2202,11 +2276,19 @@
                 <a:srgbClr val="000000"/>
               </a:solidFill>
               <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
             </a:rPr>
             <a:t>New-Fast Technology Co., LTD</a:t>
           </a:r>
+          <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:pPr algn="l" rtl="0">
@@ -2387,24 +2469,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -2412,7 +2496,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -2420,11 +2504,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -2550,24 +2642,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -2575,7 +2669,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -2583,11 +2677,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -2713,24 +2815,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -2738,7 +2842,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -2746,28 +2850,18 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
-              <a:t>New-Fast Technology Co., LT</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
-              </a:rPr>
-              <a:t>D</a:t>
+              <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:cs typeface="Times New Roman"/>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -2894,24 +2988,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -2919,7 +3015,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -2927,11 +3023,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -3057,24 +3161,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -3082,7 +3188,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -3090,11 +3196,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -3220,24 +3334,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -3245,7 +3361,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -3253,11 +3369,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -3383,24 +3507,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -3408,7 +3534,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -3416,11 +3542,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
@@ -3546,24 +3680,26 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+                <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
               </a:rPr>
               <a:t>金 兆 益 科 技 股 份 有 限 公 司</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
+            <a:endParaRPr lang="zh-TW" altLang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="-100" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
-              <a:latin typeface="標楷體" pitchFamily="65" charset="-120"/>
-              <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+              <a:latin typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:ea typeface="MingLiU" pitchFamily="54" charset="136"/>
+              <a:cs typeface="MingLiU" pitchFamily="54" charset="136"/>
             </a:endParaRPr>
           </a:p>
           <a:p>
@@ -3571,7 +3707,7 @@
               <a:lnSpc>
                 <a:spcPts val="2000"/>
               </a:lnSpc>
-              <a:defRPr sz="1000"/>
+              <a:defRPr sz="1200"/>
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
@@ -3579,11 +3715,19 @@
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="標楷體" pitchFamily="65" charset="-120"/>
+                <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                 <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               </a:rPr>
               <a:t>New-Fast Technology Co., LTD</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US" altLang="zh-TW" sz="1200" b="1" i="0" u="none" strike="noStrike" spc="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:endParaRPr>
           </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">

</xml_diff>